<commit_message>
Antes de Realizar Restructura
</commit_message>
<xml_diff>
--- a/data/BASES/INVENTARIOS.xlsx
+++ b/data/BASES/INVENTARIOS.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="138">
   <si>
     <t>CODIGO</t>
   </si>
@@ -436,6 +436,15 @@
   </si>
   <si>
     <t>36</t>
+  </si>
+  <si>
+    <t>C:\OCXRST\FOTOSPRODUCT\W2300A.jpg</t>
+  </si>
+  <si>
+    <t>2,137.51</t>
+  </si>
+  <si>
+    <t>C:\OCXRST\FOTOSPRODUCT\W2301A.JPG</t>
   </si>
 </sst>
 </file>
@@ -892,7 +901,7 @@
         <v>105</v>
       </c>
       <c r="K2" t="s">
-        <v>106</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -905,14 +914,29 @@
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2">
-        <v>2137.5100000000002</v>
+      <c r="D3" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F3" s="1">
-        <v>1</v>
+      <c r="F3" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" t="s">
+        <v>105</v>
+      </c>
+      <c r="K3" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>